<commit_message>
feat: varredura e atualizacao ate 07/10 com 68 lojas e 5550 pedidos recuperados e novos dias 05, 06 e 07/10
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-28).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-28).xlsx
@@ -935,16 +935,16 @@
     <t>214</t>
   </si>
   <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>R$ 3.006,75</t>
+    <t>26</t>
+  </si>
+  <si>
+    <t>R$ 3.009,69</t>
   </si>
   <si>
     <t>34.1</t>
   </si>
   <si>
-    <t>21.2</t>
+    <t>21.3</t>
   </si>
   <si>
     <t>4.62</t>
@@ -956,13 +956,13 @@
     <t>6.4</t>
   </si>
   <si>
-    <t>6.2</t>
-  </si>
-  <si>
-    <t>45.2%</t>
-  </si>
-  <si>
-    <t>17.1%</t>
+    <t>6.3</t>
+  </si>
+  <si>
+    <t>45.1%</t>
+  </si>
+  <si>
+    <t>16.9%</t>
   </si>
   <si>
     <t>1.8%</t>
@@ -971,25 +971,25 @@
     <t>0.2%</t>
   </si>
   <si>
-    <t>4.5%</t>
+    <t>4.4%</t>
   </si>
   <si>
     <t>1.5%</t>
   </si>
   <si>
-    <t>6.7%</t>
-  </si>
-  <si>
-    <t>2.5%</t>
-  </si>
-  <si>
-    <t>3.8%</t>
-  </si>
-  <si>
-    <t>827.0</t>
-  </si>
-  <si>
-    <t>664.0</t>
+    <t>6.6%</t>
+  </si>
+  <si>
+    <t>2.4%</t>
+  </si>
+  <si>
+    <t>3.7%</t>
+  </si>
+  <si>
+    <t>831.0</t>
+  </si>
+  <si>
+    <t>668.0</t>
   </si>
   <si>
     <t>70.0</t>
@@ -1007,13 +1007,13 @@
     <t>7.0</t>
   </si>
   <si>
-    <t>260.0</t>
+    <t>262.0</t>
   </si>
   <si>
     <t>96.0</t>
   </si>
   <si>
-    <t>146.0</t>
+    <t>148.0</t>
   </si>
   <si>
     <t>0.4%</t>
@@ -2206,7 +2206,7 @@
         <v>19507</v>
       </c>
       <c r="B6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C6" s="4">
         <v>51</v>
@@ -2236,35 +2236,93 @@
         <v>58</v>
       </c>
       <c r="L6" s="4"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="8"/>
-      <c r="S6" s="8"/>
-      <c r="T6" s="9"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="9"/>
-      <c r="X6" s="9"/>
-      <c r="Y6" s="9"/>
-      <c r="Z6" s="9"/>
-      <c r="AA6" s="9"/>
-      <c r="AB6" s="9"/>
-      <c r="AC6" s="9"/>
-      <c r="AD6" s="6"/>
-      <c r="AE6" s="6"/>
-      <c r="AF6" s="6"/>
-      <c r="AG6" s="6"/>
-      <c r="AH6" s="6"/>
-      <c r="AI6" s="6"/>
-      <c r="AJ6" s="6"/>
-      <c r="AK6" s="6"/>
-      <c r="AL6" s="6"/>
-      <c r="AM6" s="6"/>
-      <c r="AN6" s="9"/>
-      <c r="AO6" s="6"/>
+      <c r="M6" s="5">
+        <v>3844.6100000000001</v>
+      </c>
+      <c r="N6" s="6">
+        <v>41</v>
+      </c>
+      <c r="O6" s="6">
+        <v>34</v>
+      </c>
+      <c r="P6" s="7">
+        <v>5.002031707317073</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>14.933332352941177</v>
+      </c>
+      <c r="R6" s="8">
+        <v>2.8446088235294118</v>
+      </c>
+      <c r="S6" s="8">
+        <v>7</v>
+      </c>
+      <c r="T6" s="9">
+        <v>0.47058823529411764</v>
+      </c>
+      <c r="U6" s="9">
+        <v>0.029411764705882353</v>
+      </c>
+      <c r="V6" s="9">
+        <v>0</v>
+      </c>
+      <c r="W6" s="9">
+        <v>0</v>
+      </c>
+      <c r="X6" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="9">
+        <v>0.029411764705882353</v>
+      </c>
+      <c r="AB6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="6">
+        <v>1</v>
+      </c>
+      <c r="AE6" s="6">
+        <v>1</v>
+      </c>
+      <c r="AF6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK6" s="6">
+        <v>1</v>
+      </c>
+      <c r="AL6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO6" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP6" s="4">
         <v>58</v>
       </c>
@@ -7143,7 +7201,7 @@
         <v>4.9729187499999998</v>
       </c>
       <c r="S38" s="8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T38" s="9">
         <v>0.3888888888888889</v>
@@ -25036,7 +25094,7 @@
         <v>19859</v>
       </c>
       <c r="B158" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C158" s="4">
         <v>51</v>
@@ -25066,35 +25124,93 @@
         <v>58</v>
       </c>
       <c r="L158" s="4"/>
-      <c r="M158" s="5"/>
-      <c r="N158" s="6"/>
-      <c r="O158" s="6"/>
-      <c r="P158" s="7"/>
-      <c r="Q158" s="8"/>
-      <c r="R158" s="8"/>
-      <c r="S158" s="8"/>
-      <c r="T158" s="9"/>
-      <c r="U158" s="9"/>
-      <c r="V158" s="9"/>
-      <c r="W158" s="9"/>
-      <c r="X158" s="9"/>
-      <c r="Y158" s="9"/>
-      <c r="Z158" s="9"/>
-      <c r="AA158" s="9"/>
-      <c r="AB158" s="9"/>
-      <c r="AC158" s="9"/>
-      <c r="AD158" s="6"/>
-      <c r="AE158" s="6"/>
-      <c r="AF158" s="6"/>
-      <c r="AG158" s="6"/>
-      <c r="AH158" s="6"/>
-      <c r="AI158" s="6"/>
-      <c r="AJ158" s="6"/>
-      <c r="AK158" s="6"/>
-      <c r="AL158" s="6"/>
-      <c r="AM158" s="6"/>
-      <c r="AN158" s="9"/>
-      <c r="AO158" s="6"/>
+      <c r="M158" s="5">
+        <v>2714.4499999999998</v>
+      </c>
+      <c r="N158" s="6">
+        <v>25</v>
+      </c>
+      <c r="O158" s="6">
+        <v>20</v>
+      </c>
+      <c r="P158" s="7">
+        <v>4.6724346153846152</v>
+      </c>
+      <c r="Q158" s="8">
+        <v>14.925835000000001</v>
+      </c>
+      <c r="R158" s="8">
+        <v>3.206142105263158</v>
+      </c>
+      <c r="S158" s="8">
+        <v>7</v>
+      </c>
+      <c r="T158" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U158" s="9">
+        <v>0.050000000000000003</v>
+      </c>
+      <c r="V158" s="9">
+        <v>0</v>
+      </c>
+      <c r="W158" s="9">
+        <v>0</v>
+      </c>
+      <c r="X158" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y158" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z158" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA158" s="9">
+        <v>0.050000000000000003</v>
+      </c>
+      <c r="AB158" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC158" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD158" s="6">
+        <v>1</v>
+      </c>
+      <c r="AE158" s="6">
+        <v>1</v>
+      </c>
+      <c r="AF158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK158" s="6">
+        <v>1</v>
+      </c>
+      <c r="AL158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN158" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO158" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP158" s="4">
         <v>58</v>
       </c>
@@ -30585,7 +30701,9 @@
       <c r="N195" s="6">
         <v>37</v>
       </c>
-      <c r="O195" s="6"/>
+      <c r="O195" s="6">
+        <v>18</v>
+      </c>
       <c r="P195" s="7">
         <v>4.0779411764705884</v>
       </c>
@@ -30595,31 +30713,75 @@
       <c r="R195" s="8">
         <v>4.2666666666666666</v>
       </c>
-      <c r="S195" s="8"/>
+      <c r="S195" s="8">
+        <v>7</v>
+      </c>
       <c r="T195" s="9">
         <v>0.44444444444444442</v>
       </c>
-      <c r="U195" s="9"/>
-      <c r="V195" s="9"/>
-      <c r="W195" s="9"/>
-      <c r="X195" s="9"/>
-      <c r="Y195" s="9"/>
-      <c r="Z195" s="9"/>
-      <c r="AA195" s="9"/>
-      <c r="AB195" s="9"/>
-      <c r="AC195" s="9"/>
-      <c r="AD195" s="6"/>
-      <c r="AE195" s="6"/>
-      <c r="AF195" s="6"/>
-      <c r="AG195" s="6"/>
-      <c r="AH195" s="6"/>
-      <c r="AI195" s="6"/>
-      <c r="AJ195" s="6"/>
-      <c r="AK195" s="6"/>
-      <c r="AL195" s="6"/>
-      <c r="AM195" s="6"/>
-      <c r="AN195" s="9"/>
-      <c r="AO195" s="6"/>
+      <c r="U195" s="9">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="V195" s="9">
+        <v>0</v>
+      </c>
+      <c r="W195" s="9">
+        <v>0</v>
+      </c>
+      <c r="X195" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y195" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC195" s="9">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="AD195" s="6">
+        <v>2</v>
+      </c>
+      <c r="AE195" s="6">
+        <v>2</v>
+      </c>
+      <c r="AF195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM195" s="6">
+        <v>2</v>
+      </c>
+      <c r="AN195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO195" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP195" s="4">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
feat: rotacao de semanas para 21 a 27, 28 a 04, 05 a 11 e 12 a 14 com 54 lojas e 4075 pedidos resgatados
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-28).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-28).xlsx
@@ -932,22 +932,25 @@
     <t>GUIMARAES FRAGA,MARESSA</t>
   </si>
   <si>
-    <t>214</t>
+    <t>DE LOURDES RAMOS,MARIA</t>
+  </si>
+  <si>
+    <t>215</t>
   </si>
   <si>
     <t>26</t>
   </si>
   <si>
-    <t>R$ 3.009,69</t>
+    <t>R$ 2.999,42</t>
   </si>
   <si>
-    <t>34.1</t>
+    <t>34.0</t>
   </si>
   <si>
-    <t>21.3</t>
+    <t>21.2</t>
   </si>
   <si>
-    <t>4.62</t>
+    <t>4.61</t>
   </si>
   <si>
     <t>17.8</t>
@@ -959,7 +962,7 @@
     <t>6.3</t>
   </si>
   <si>
-    <t>45.1%</t>
+    <t>44.8%</t>
   </si>
   <si>
     <t>16.9%</t>
@@ -977,7 +980,7 @@
     <t>1.5%</t>
   </si>
   <si>
-    <t>6.6%</t>
+    <t>6.7%</t>
   </si>
   <si>
     <t>2.4%</t>
@@ -986,31 +989,31 @@
     <t>3.7%</t>
   </si>
   <si>
-    <t>831.0</t>
+    <t>848.0</t>
   </si>
   <si>
-    <t>668.0</t>
+    <t>678.0</t>
   </si>
   <si>
-    <t>70.0</t>
+    <t>71.0</t>
   </si>
   <si>
     <t>9.0</t>
   </si>
   <si>
-    <t>173.0</t>
+    <t>178.0</t>
   </si>
   <si>
-    <t>58.0</t>
+    <t>60.0</t>
   </si>
   <si>
-    <t>7.0</t>
+    <t>8.0</t>
   </si>
   <si>
-    <t>262.0</t>
+    <t>267.0</t>
   </si>
   <si>
-    <t>96.0</t>
+    <t>98.0</t>
   </si>
   <si>
     <t>148.0</t>
@@ -1019,7 +1022,7 @@
     <t>0.4%</t>
   </si>
   <si>
-    <t>17.0</t>
+    <t>18.0</t>
   </si>
   <si>
     <t>1</t>
@@ -18840,33 +18843,79 @@
       <c r="L116" s="4"/>
       <c r="M116" s="5"/>
       <c r="N116" s="6"/>
-      <c r="O116" s="6"/>
+      <c r="O116" s="6">
+        <v>13</v>
+      </c>
       <c r="P116" s="7"/>
       <c r="Q116" s="8"/>
       <c r="R116" s="8"/>
-      <c r="S116" s="8"/>
+      <c r="S116" s="8">
+        <v>7</v>
+      </c>
       <c r="T116" s="9"/>
-      <c r="U116" s="9"/>
-      <c r="V116" s="9"/>
-      <c r="W116" s="9"/>
-      <c r="X116" s="9"/>
-      <c r="Y116" s="9"/>
-      <c r="Z116" s="9"/>
-      <c r="AA116" s="9"/>
-      <c r="AB116" s="9"/>
-      <c r="AC116" s="9"/>
-      <c r="AD116" s="6"/>
-      <c r="AE116" s="6"/>
-      <c r="AF116" s="6"/>
-      <c r="AG116" s="6"/>
-      <c r="AH116" s="6"/>
-      <c r="AI116" s="6"/>
-      <c r="AJ116" s="6"/>
-      <c r="AK116" s="6"/>
-      <c r="AL116" s="6"/>
-      <c r="AM116" s="6"/>
-      <c r="AN116" s="9"/>
-      <c r="AO116" s="6"/>
+      <c r="U116" s="9">
+        <v>0.23076923076923078</v>
+      </c>
+      <c r="V116" s="9">
+        <v>0</v>
+      </c>
+      <c r="W116" s="9">
+        <v>0</v>
+      </c>
+      <c r="X116" s="9">
+        <v>0.076923076923076927</v>
+      </c>
+      <c r="Y116" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z116" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA116" s="9">
+        <v>0.076923076923076927</v>
+      </c>
+      <c r="AB116" s="9">
+        <v>0.076923076923076927</v>
+      </c>
+      <c r="AC116" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD116" s="6">
+        <v>3</v>
+      </c>
+      <c r="AE116" s="6">
+        <v>3</v>
+      </c>
+      <c r="AF116" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG116" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH116" s="6">
+        <v>1</v>
+      </c>
+      <c r="AI116" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ116" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK116" s="6">
+        <v>1</v>
+      </c>
+      <c r="AL116" s="6">
+        <v>1</v>
+      </c>
+      <c r="AM116" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN116" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO116" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP116" s="4">
         <v>58</v>
       </c>
@@ -22607,7 +22656,7 @@
         <v>19793</v>
       </c>
       <c r="B141" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C141" s="4">
         <v>51</v>
@@ -22637,35 +22686,93 @@
         <v>58</v>
       </c>
       <c r="L141" s="4"/>
-      <c r="M141" s="5"/>
-      <c r="N141" s="6"/>
-      <c r="O141" s="6"/>
-      <c r="P141" s="7"/>
-      <c r="Q141" s="8"/>
-      <c r="R141" s="8"/>
-      <c r="S141" s="8"/>
-      <c r="T141" s="9"/>
-      <c r="U141" s="9"/>
-      <c r="V141" s="9"/>
-      <c r="W141" s="9"/>
-      <c r="X141" s="9"/>
-      <c r="Y141" s="9"/>
-      <c r="Z141" s="9"/>
-      <c r="AA141" s="9"/>
-      <c r="AB141" s="9"/>
-      <c r="AC141" s="9"/>
-      <c r="AD141" s="6"/>
-      <c r="AE141" s="6"/>
-      <c r="AF141" s="6"/>
-      <c r="AG141" s="6"/>
-      <c r="AH141" s="6"/>
-      <c r="AI141" s="6"/>
-      <c r="AJ141" s="6"/>
-      <c r="AK141" s="6"/>
-      <c r="AL141" s="6"/>
-      <c r="AM141" s="6"/>
-      <c r="AN141" s="9"/>
-      <c r="AO141" s="6"/>
+      <c r="M141" s="5">
+        <v>1089.1600000000001</v>
+      </c>
+      <c r="N141" s="6">
+        <v>17</v>
+      </c>
+      <c r="O141" s="6">
+        <v>14</v>
+      </c>
+      <c r="P141" s="7">
+        <v>2.2607823529411766</v>
+      </c>
+      <c r="Q141" s="8">
+        <v>12.440478571428571</v>
+      </c>
+      <c r="R141" s="8">
+        <v>2.0714285714285716</v>
+      </c>
+      <c r="S141" s="8">
+        <v>8</v>
+      </c>
+      <c r="T141" s="9">
+        <v>0.9285714285714286</v>
+      </c>
+      <c r="U141" s="9">
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="V141" s="9">
+        <v>0</v>
+      </c>
+      <c r="W141" s="9">
+        <v>0</v>
+      </c>
+      <c r="X141" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y141" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z141" s="9">
+        <v>0.071428571428571425</v>
+      </c>
+      <c r="AA141" s="9">
+        <v>0.071428571428571425</v>
+      </c>
+      <c r="AB141" s="9">
+        <v>0.071428571428571425</v>
+      </c>
+      <c r="AC141" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD141" s="6">
+        <v>3</v>
+      </c>
+      <c r="AE141" s="6">
+        <v>2</v>
+      </c>
+      <c r="AF141" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG141" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH141" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI141" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ141" s="6">
+        <v>1</v>
+      </c>
+      <c r="AK141" s="6">
+        <v>1</v>
+      </c>
+      <c r="AL141" s="6">
+        <v>1</v>
+      </c>
+      <c r="AM141" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN141" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO141" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP141" s="4">
         <v>58</v>
       </c>
@@ -33492,137 +33599,282 @@
       </c>
     </row>
     <row r="216" ht="13.5" customHeight="1">
-      <c t="s" r="A216" s="11">
+      <c r="A216" s="2">
+        <v>19980</v>
+      </c>
+      <c r="B216" s="3">
+        <v>-1</v>
+      </c>
+      <c t="s" r="C216" s="4">
+        <v>51</v>
+      </c>
+      <c t="s" r="D216" s="4">
+        <v>52</v>
+      </c>
+      <c t="s" r="E216" s="4">
+        <v>53</v>
+      </c>
+      <c t="s" r="F216" s="4">
+        <v>54</v>
+      </c>
+      <c t="s" r="G216" s="4">
+        <v>55</v>
+      </c>
+      <c t="s" r="H216" s="4">
+        <v>56</v>
+      </c>
+      <c t="s" r="I216" s="4">
+        <v>57</v>
+      </c>
+      <c t="s" r="J216" s="4">
+        <v>54</v>
+      </c>
+      <c t="s" r="K216" s="4">
+        <v>58</v>
+      </c>
+      <c r="L216" s="4"/>
+      <c r="M216" s="5"/>
+      <c r="N216" s="6"/>
+      <c r="O216" s="6">
+        <v>21</v>
+      </c>
+      <c r="P216" s="7"/>
+      <c r="Q216" s="8"/>
+      <c r="R216" s="8"/>
+      <c r="S216" s="8">
+        <v>7</v>
+      </c>
+      <c r="T216" s="9"/>
+      <c r="U216" s="9">
+        <v>0.23809523809523808</v>
+      </c>
+      <c r="V216" s="9">
+        <v>0.047619047619047616</v>
+      </c>
+      <c r="W216" s="9">
+        <v>0</v>
+      </c>
+      <c r="X216" s="9">
+        <v>0.19047619047619047</v>
+      </c>
+      <c r="Y216" s="9">
+        <v>0.095238095238095233</v>
+      </c>
+      <c r="Z216" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA216" s="9">
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="AB216" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC216" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD216" s="6">
+        <v>11</v>
+      </c>
+      <c r="AE216" s="6">
+        <v>5</v>
+      </c>
+      <c r="AF216" s="6">
+        <v>1</v>
+      </c>
+      <c r="AG216" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH216" s="6">
+        <v>4</v>
+      </c>
+      <c r="AI216" s="6">
+        <v>2</v>
+      </c>
+      <c r="AJ216" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK216" s="6">
+        <v>3</v>
+      </c>
+      <c r="AL216" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM216" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN216" s="9">
+        <v>0.047619047619047616</v>
+      </c>
+      <c r="AO216" s="6">
+        <v>1</v>
+      </c>
+      <c t="s" r="AP216" s="4">
+        <v>58</v>
+      </c>
+      <c t="s" r="AQ216" s="4">
+        <v>59</v>
+      </c>
+      <c t="s" r="AR216" s="4">
         <v>307</v>
       </c>
-      <c t="s" r="B216" s="11">
+      <c t="s" r="AS216" s="4">
+        <v>60</v>
+      </c>
+      <c t="s" r="AT216" s="4">
+        <v>61</v>
+      </c>
+      <c t="s" r="AU216" s="4">
+        <v>62</v>
+      </c>
+      <c t="s" r="AV216" s="4">
+        <v>59</v>
+      </c>
+      <c t="s" r="AW216" s="4">
+        <v>59</v>
+      </c>
+      <c r="AX216" s="2">
+        <v>1</v>
+      </c>
+      <c r="AY216" s="2">
+        <v>1</v>
+      </c>
+      <c r="AZ216" s="10"/>
+      <c t="s" r="BA216" s="4">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="217" ht="13.5" customHeight="1">
+      <c t="s" r="A217" s="11">
         <v>308</v>
       </c>
-      <c r="C216" s="12"/>
-      <c r="D216" s="12"/>
-      <c r="E216" s="12"/>
-      <c r="F216" s="12"/>
-      <c r="G216" s="12"/>
-      <c r="H216" s="12"/>
-      <c r="I216" s="12"/>
-      <c r="J216" s="12"/>
-      <c r="K216" s="12"/>
-      <c r="L216" s="12"/>
-      <c t="s" r="M216" s="11">
+      <c t="s" r="B217" s="11">
         <v>309</v>
       </c>
-      <c t="s" r="N216" s="11">
+      <c r="C217" s="12"/>
+      <c r="D217" s="12"/>
+      <c r="E217" s="12"/>
+      <c r="F217" s="12"/>
+      <c r="G217" s="12"/>
+      <c r="H217" s="12"/>
+      <c r="I217" s="12"/>
+      <c r="J217" s="12"/>
+      <c r="K217" s="12"/>
+      <c r="L217" s="12"/>
+      <c t="s" r="M217" s="11">
         <v>310</v>
       </c>
-      <c t="s" r="O216" s="11">
+      <c t="s" r="N217" s="11">
         <v>311</v>
       </c>
-      <c t="s" r="P216" s="11">
+      <c t="s" r="O217" s="11">
         <v>312</v>
       </c>
-      <c t="s" r="Q216" s="11">
+      <c t="s" r="P217" s="11">
         <v>313</v>
       </c>
-      <c t="s" r="R216" s="11">
+      <c t="s" r="Q217" s="11">
         <v>314</v>
       </c>
-      <c t="s" r="S216" s="11">
+      <c t="s" r="R217" s="11">
         <v>315</v>
       </c>
-      <c t="s" r="T216" s="11">
+      <c t="s" r="S217" s="11">
         <v>316</v>
       </c>
-      <c t="s" r="U216" s="11">
+      <c t="s" r="T217" s="11">
         <v>317</v>
       </c>
-      <c t="s" r="V216" s="11">
+      <c t="s" r="U217" s="11">
         <v>318</v>
       </c>
-      <c t="s" r="W216" s="11">
+      <c t="s" r="V217" s="11">
         <v>319</v>
       </c>
-      <c t="s" r="X216" s="11">
+      <c t="s" r="W217" s="11">
         <v>320</v>
       </c>
-      <c t="s" r="Y216" s="11">
+      <c t="s" r="X217" s="11">
         <v>321</v>
       </c>
-      <c t="s" r="Z216" s="11">
-        <v>319</v>
-      </c>
-      <c t="s" r="AA216" s="11">
+      <c t="s" r="Y217" s="11">
         <v>322</v>
       </c>
-      <c t="s" r="AB216" s="11">
+      <c t="s" r="Z217" s="11">
+        <v>320</v>
+      </c>
+      <c t="s" r="AA217" s="11">
         <v>323</v>
       </c>
-      <c t="s" r="AC216" s="11">
+      <c t="s" r="AB217" s="11">
         <v>324</v>
       </c>
-      <c t="s" r="AD216" s="11">
+      <c t="s" r="AC217" s="11">
         <v>325</v>
       </c>
-      <c t="s" r="AE216" s="11">
+      <c t="s" r="AD217" s="11">
         <v>326</v>
       </c>
-      <c t="s" r="AF216" s="11">
+      <c t="s" r="AE217" s="11">
         <v>327</v>
       </c>
-      <c t="s" r="AG216" s="11">
+      <c t="s" r="AF217" s="11">
         <v>328</v>
       </c>
-      <c t="s" r="AH216" s="11">
+      <c t="s" r="AG217" s="11">
         <v>329</v>
       </c>
-      <c t="s" r="AI216" s="11">
+      <c t="s" r="AH217" s="11">
         <v>330</v>
       </c>
-      <c t="s" r="AJ216" s="11">
+      <c t="s" r="AI217" s="11">
         <v>331</v>
       </c>
-      <c t="s" r="AK216" s="11">
+      <c t="s" r="AJ217" s="11">
         <v>332</v>
       </c>
-      <c t="s" r="AL216" s="11">
+      <c t="s" r="AK217" s="11">
         <v>333</v>
       </c>
-      <c t="s" r="AM216" s="11">
+      <c t="s" r="AL217" s="11">
         <v>334</v>
       </c>
-      <c t="s" r="AN216" s="11">
+      <c t="s" r="AM217" s="11">
         <v>335</v>
       </c>
-      <c t="s" r="AO216" s="11">
+      <c t="s" r="AN217" s="11">
         <v>336</v>
       </c>
-      <c r="AP216" s="12"/>
-      <c t="s" r="AQ216" s="12">
-        <v>59</v>
-      </c>
-      <c r="AR216" s="12"/>
-      <c r="AS216" s="12"/>
-      <c r="AT216" s="12"/>
-      <c r="AU216" s="12"/>
-      <c t="s" r="AV216" s="12">
-        <v>59</v>
-      </c>
-      <c t="s" r="AW216" s="12">
-        <v>59</v>
-      </c>
-      <c t="s" r="AX216" s="11">
+      <c t="s" r="AO217" s="11">
         <v>337</v>
       </c>
-      <c t="s" r="AY216" s="11">
-        <v>337</v>
-      </c>
-      <c r="AZ216" s="12"/>
-      <c r="BA216" s="12"/>
+      <c r="AP217" s="12"/>
+      <c t="s" r="AQ217" s="12">
+        <v>59</v>
+      </c>
+      <c r="AR217" s="12"/>
+      <c r="AS217" s="12"/>
+      <c r="AT217" s="12"/>
+      <c r="AU217" s="12"/>
+      <c t="s" r="AV217" s="12">
+        <v>59</v>
+      </c>
+      <c t="s" r="AW217" s="12">
+        <v>59</v>
+      </c>
+      <c t="s" r="AX217" s="11">
+        <v>338</v>
+      </c>
+      <c t="s" r="AY217" s="11">
+        <v>338</v>
+      </c>
+      <c r="AZ217" s="12"/>
+      <c r="BA217" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:BA216" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:BA217" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>